<commit_message>
Conexión de la página con el inventario en Google Sheets
- apps-script/Codigo.gs: aplicación web que entrega el stock (disponible,
  estado, precio, visible) y registra cada pedido como Pendiente en Pedidos
  y Detalle, sin tocar fórmulas, sin duplicar y descartando SKUs inexistentes.
- index.html: envía cupón y descripción limpia (con las elecciones del combo).
- Inventario: instrucciones actualizadas (precios de la hoja mandan, combos,
  cupones en Notas, conexión con la página).
- CONECTAR-INVENTARIO.txt: pasos para publicar el script y pegar la URL.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vfZoR2jzny9XDHVyMdLYu
</commit_message>
<xml_diff>
--- a/inventario-wings-zone.xlsx
+++ b/inventario-wings-zone.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A27"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="120" customWidth="1" style="18" min="1" max="1"/>
@@ -543,6 +543,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="19">
       <c r="A3" s="21" t="inlineStr">
         <is>
@@ -677,7 +678,7 @@
     <row r="24" ht="15" customHeight="1" s="19">
       <c r="A24" s="22" t="inlineStr">
         <is>
-          <t>- Los precios salen del menú de OlaClick consultado el 14/10/2026. Si cambias un precio allá, cámbialo aquí también.</t>
+          <t>- Los precios de la hoja Inventario mandan: si la página está conectada, muestra el precio de aquí. Si cambias un precio, cámbialo solo aquí.</t>
         </is>
       </c>
     </row>
@@ -691,7 +692,7 @@
     <row r="26" ht="15" customHeight="1" s="19">
       <c r="A26" s="22" t="inlineStr">
         <is>
-          <t>- Los combos se cuentan como unidades vendibles. No descuentan ingredientes sueltos (alitas, papas, empaques).</t>
+          <t>- Los combos se cuentan como unidades vendibles. La salsa y los acompañamientos que elige el cliente van en la descripción del pedido y no descuentan stock de Adicionales.</t>
         </is>
       </c>
     </row>
@@ -699,6 +700,56 @@
       <c r="A27" s="22" t="inlineStr">
         <is>
           <t>- Las fórmulas de las hojas Pedidos y Detalle están listas hasta la fila 300. Si pasas de ahí, copia la última fila hacia abajo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28"/>
+    <row r="29">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>Conexión con la página web</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="22" t="inlineStr">
+        <is>
+          <t>- La página lee de la hoja Inventario el disponible, el estado, el precio y si el producto es visible (columna "Visible en página": Sí/No).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
+        <is>
+          <t>- Cada pedido enviado desde la página llega solo a Pedidos (estado Pendiente) y a Detalle (un renglón por producto). Sus unidades quedan reservadas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="22" t="inlineStr">
+        <is>
+          <t>- Revisa el pedido en WhatsApp, escribe el valor del domicilio en la columna Domicilio y cambia el estado a Confirmado (descuenta stock) o Cancelado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="22" t="inlineStr">
+        <is>
+          <t>- Si el cliente usó un cupón, aparece en la columna Notas. Los de primera compra dicen "verificar": revisa que sea su primer pedido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="22" t="inlineStr">
+        <is>
+          <t>- Para agregar un producto nuevo: añade su fila en Inventario con el mismo SKU que tiene en la página.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="22" t="inlineStr">
+        <is>
+          <t>- Los pasos para conectar están en el archivo CONECTAR-INVENTARIO.txt.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Reseñas de clientes desde la hoja de Google
- Apps Script: GET ?action=reviews devuelve las reseñas con Publicar = Sí
  (máx. 12, más recientes primero) y crea la hoja Reseñas si no existe.
- Página: sección 'Lo que dicen nuestros clientes' con estrellas, promedio,
  nombre e inicial del apellido; oculta si no hay reseñas publicadas.
- Inventario (.xlsx): hoja Reseñas e instrucciones; guía de conexión actualizada.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014vfZoR2jzny9XDHVyMdLYu
</commit_message>
<xml_diff>
--- a/inventario-wings-zone.xlsx
+++ b/inventario-wings-zone.xlsx
@@ -13,6 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Pedidos" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Detalle" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Movimientos" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Reseñas" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -21,12 +22,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy\ hh:mm"/>
     <numFmt numFmtId="166" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="167" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <charset val="1"/>
@@ -92,8 +94,19 @@
       <color rgb="FF0000FF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <color rgb="000000FF"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -110,6 +123,16 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
         <bgColor rgb="FFFFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001A1A1A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -147,7 +170,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -254,6 +277,13 @@
     <xf numFmtId="166" fontId="9" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -530,7 +560,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:A35"/>
+  <dimension ref="A1:A40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="120" customWidth="1" style="18" min="1" max="1"/>
@@ -543,7 +573,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3" ht="15" customHeight="1" s="19">
       <c r="A3" s="21" t="inlineStr">
         <is>
@@ -703,7 +732,6 @@
         </is>
       </c>
     </row>
-    <row r="28"/>
     <row r="29">
       <c r="A29" s="21" t="inlineStr">
         <is>
@@ -750,6 +778,35 @@
       <c r="A35" s="22" t="inlineStr">
         <is>
           <t>- Los pasos para conectar están en el archivo CONECTAR-INVENTARIO.txt.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="21" t="inlineStr">
+        <is>
+          <t>Reseñas</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="22" t="inlineStr">
+        <is>
+          <t>- En la hoja Reseñas escribe las opiniones de tus clientes: nombre, estrellas (1 a 5), comentario y fecha.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="22" t="inlineStr">
+        <is>
+          <t>- Solo aparecen en la página las que tengan Sí en Publicar (máximo las 12 más recientes). Usa solo opiniones reales y con permiso del cliente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="22" t="inlineStr">
+        <is>
+          <t>- La página muestra el nombre y la inicial del apellido (Laura Martínez -&gt; Laura M.).</t>
         </is>
       </c>
     </row>
@@ -26760,4 +26817,774 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="portrait" paperSize="9" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver" blackAndWhite="0" draft="0" horizontalDpi="300" verticalDpi="300" copies="1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E104"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" style="19" min="1" max="1"/>
+    <col width="16" customWidth="1" style="19" min="2" max="2"/>
+    <col width="70" customWidth="1" style="19" min="3" max="3"/>
+    <col width="13" customWidth="1" style="19" min="4" max="4"/>
+    <col width="11" customWidth="1" style="19" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="36" t="inlineStr">
+        <is>
+          <t>Reseñas de clientes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Un renglón por opinión. Solo se muestran en la página las que tengan Sí en Publicar. Usa nombre e inicial del apellido (ej: Laura M.).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="37" t="inlineStr">
+        <is>
+          <t>Nombre</t>
+        </is>
+      </c>
+      <c r="B4" s="37" t="inlineStr">
+        <is>
+          <t>Estrellas (1 a 5)</t>
+        </is>
+      </c>
+      <c r="C4" s="37" t="inlineStr">
+        <is>
+          <t>Comentario</t>
+        </is>
+      </c>
+      <c r="D4" s="37" t="inlineStr">
+        <is>
+          <t>Fecha</t>
+        </is>
+      </c>
+      <c r="E4" s="37" t="inlineStr">
+        <is>
+          <t>Publicar</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="38" t="n"/>
+      <c r="B5" s="38" t="n"/>
+      <c r="C5" s="39" t="n"/>
+      <c r="D5" s="40" t="n"/>
+      <c r="E5" s="38" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="38" t="n"/>
+      <c r="B6" s="38" t="n"/>
+      <c r="C6" s="39" t="n"/>
+      <c r="D6" s="40" t="n"/>
+      <c r="E6" s="38" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="38" t="n"/>
+      <c r="B7" s="38" t="n"/>
+      <c r="C7" s="39" t="n"/>
+      <c r="D7" s="40" t="n"/>
+      <c r="E7" s="38" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="38" t="n"/>
+      <c r="B8" s="38" t="n"/>
+      <c r="C8" s="39" t="n"/>
+      <c r="D8" s="40" t="n"/>
+      <c r="E8" s="38" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="38" t="n"/>
+      <c r="B9" s="38" t="n"/>
+      <c r="C9" s="39" t="n"/>
+      <c r="D9" s="40" t="n"/>
+      <c r="E9" s="38" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="38" t="n"/>
+      <c r="B10" s="38" t="n"/>
+      <c r="C10" s="39" t="n"/>
+      <c r="D10" s="40" t="n"/>
+      <c r="E10" s="38" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="38" t="n"/>
+      <c r="B11" s="38" t="n"/>
+      <c r="C11" s="39" t="n"/>
+      <c r="D11" s="40" t="n"/>
+      <c r="E11" s="38" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="38" t="n"/>
+      <c r="B12" s="38" t="n"/>
+      <c r="C12" s="39" t="n"/>
+      <c r="D12" s="40" t="n"/>
+      <c r="E12" s="38" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="38" t="n"/>
+      <c r="B13" s="38" t="n"/>
+      <c r="C13" s="39" t="n"/>
+      <c r="D13" s="40" t="n"/>
+      <c r="E13" s="38" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="38" t="n"/>
+      <c r="B14" s="38" t="n"/>
+      <c r="C14" s="39" t="n"/>
+      <c r="D14" s="40" t="n"/>
+      <c r="E14" s="38" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="38" t="n"/>
+      <c r="B15" s="38" t="n"/>
+      <c r="C15" s="39" t="n"/>
+      <c r="D15" s="40" t="n"/>
+      <c r="E15" s="38" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="38" t="n"/>
+      <c r="B16" s="38" t="n"/>
+      <c r="C16" s="39" t="n"/>
+      <c r="D16" s="40" t="n"/>
+      <c r="E16" s="38" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="38" t="n"/>
+      <c r="B17" s="38" t="n"/>
+      <c r="C17" s="39" t="n"/>
+      <c r="D17" s="40" t="n"/>
+      <c r="E17" s="38" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="38" t="n"/>
+      <c r="B18" s="38" t="n"/>
+      <c r="C18" s="39" t="n"/>
+      <c r="D18" s="40" t="n"/>
+      <c r="E18" s="38" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="38" t="n"/>
+      <c r="B19" s="38" t="n"/>
+      <c r="C19" s="39" t="n"/>
+      <c r="D19" s="40" t="n"/>
+      <c r="E19" s="38" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="38" t="n"/>
+      <c r="B20" s="38" t="n"/>
+      <c r="C20" s="39" t="n"/>
+      <c r="D20" s="40" t="n"/>
+      <c r="E20" s="38" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="38" t="n"/>
+      <c r="B21" s="38" t="n"/>
+      <c r="C21" s="39" t="n"/>
+      <c r="D21" s="40" t="n"/>
+      <c r="E21" s="38" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="38" t="n"/>
+      <c r="B22" s="38" t="n"/>
+      <c r="C22" s="39" t="n"/>
+      <c r="D22" s="40" t="n"/>
+      <c r="E22" s="38" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="38" t="n"/>
+      <c r="B23" s="38" t="n"/>
+      <c r="C23" s="39" t="n"/>
+      <c r="D23" s="40" t="n"/>
+      <c r="E23" s="38" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="38" t="n"/>
+      <c r="B24" s="38" t="n"/>
+      <c r="C24" s="39" t="n"/>
+      <c r="D24" s="40" t="n"/>
+      <c r="E24" s="38" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="38" t="n"/>
+      <c r="B25" s="38" t="n"/>
+      <c r="C25" s="39" t="n"/>
+      <c r="D25" s="40" t="n"/>
+      <c r="E25" s="38" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="38" t="n"/>
+      <c r="B26" s="38" t="n"/>
+      <c r="C26" s="39" t="n"/>
+      <c r="D26" s="40" t="n"/>
+      <c r="E26" s="38" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="38" t="n"/>
+      <c r="B27" s="38" t="n"/>
+      <c r="C27" s="39" t="n"/>
+      <c r="D27" s="40" t="n"/>
+      <c r="E27" s="38" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="38" t="n"/>
+      <c r="B28" s="38" t="n"/>
+      <c r="C28" s="39" t="n"/>
+      <c r="D28" s="40" t="n"/>
+      <c r="E28" s="38" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="38" t="n"/>
+      <c r="B29" s="38" t="n"/>
+      <c r="C29" s="39" t="n"/>
+      <c r="D29" s="40" t="n"/>
+      <c r="E29" s="38" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="38" t="n"/>
+      <c r="B30" s="38" t="n"/>
+      <c r="C30" s="39" t="n"/>
+      <c r="D30" s="40" t="n"/>
+      <c r="E30" s="38" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="38" t="n"/>
+      <c r="B31" s="38" t="n"/>
+      <c r="C31" s="39" t="n"/>
+      <c r="D31" s="40" t="n"/>
+      <c r="E31" s="38" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="38" t="n"/>
+      <c r="B32" s="38" t="n"/>
+      <c r="C32" s="39" t="n"/>
+      <c r="D32" s="40" t="n"/>
+      <c r="E32" s="38" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="38" t="n"/>
+      <c r="B33" s="38" t="n"/>
+      <c r="C33" s="39" t="n"/>
+      <c r="D33" s="40" t="n"/>
+      <c r="E33" s="38" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="38" t="n"/>
+      <c r="B34" s="38" t="n"/>
+      <c r="C34" s="39" t="n"/>
+      <c r="D34" s="40" t="n"/>
+      <c r="E34" s="38" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="38" t="n"/>
+      <c r="B35" s="38" t="n"/>
+      <c r="C35" s="39" t="n"/>
+      <c r="D35" s="40" t="n"/>
+      <c r="E35" s="38" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="38" t="n"/>
+      <c r="B36" s="38" t="n"/>
+      <c r="C36" s="39" t="n"/>
+      <c r="D36" s="40" t="n"/>
+      <c r="E36" s="38" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="38" t="n"/>
+      <c r="B37" s="38" t="n"/>
+      <c r="C37" s="39" t="n"/>
+      <c r="D37" s="40" t="n"/>
+      <c r="E37" s="38" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="38" t="n"/>
+      <c r="B38" s="38" t="n"/>
+      <c r="C38" s="39" t="n"/>
+      <c r="D38" s="40" t="n"/>
+      <c r="E38" s="38" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="38" t="n"/>
+      <c r="B39" s="38" t="n"/>
+      <c r="C39" s="39" t="n"/>
+      <c r="D39" s="40" t="n"/>
+      <c r="E39" s="38" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="38" t="n"/>
+      <c r="B40" s="38" t="n"/>
+      <c r="C40" s="39" t="n"/>
+      <c r="D40" s="40" t="n"/>
+      <c r="E40" s="38" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="38" t="n"/>
+      <c r="B41" s="38" t="n"/>
+      <c r="C41" s="39" t="n"/>
+      <c r="D41" s="40" t="n"/>
+      <c r="E41" s="38" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="38" t="n"/>
+      <c r="B42" s="38" t="n"/>
+      <c r="C42" s="39" t="n"/>
+      <c r="D42" s="40" t="n"/>
+      <c r="E42" s="38" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="38" t="n"/>
+      <c r="B43" s="38" t="n"/>
+      <c r="C43" s="39" t="n"/>
+      <c r="D43" s="40" t="n"/>
+      <c r="E43" s="38" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="38" t="n"/>
+      <c r="B44" s="38" t="n"/>
+      <c r="C44" s="39" t="n"/>
+      <c r="D44" s="40" t="n"/>
+      <c r="E44" s="38" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="38" t="n"/>
+      <c r="B45" s="38" t="n"/>
+      <c r="C45" s="39" t="n"/>
+      <c r="D45" s="40" t="n"/>
+      <c r="E45" s="38" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="38" t="n"/>
+      <c r="B46" s="38" t="n"/>
+      <c r="C46" s="39" t="n"/>
+      <c r="D46" s="40" t="n"/>
+      <c r="E46" s="38" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="38" t="n"/>
+      <c r="B47" s="38" t="n"/>
+      <c r="C47" s="39" t="n"/>
+      <c r="D47" s="40" t="n"/>
+      <c r="E47" s="38" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="38" t="n"/>
+      <c r="B48" s="38" t="n"/>
+      <c r="C48" s="39" t="n"/>
+      <c r="D48" s="40" t="n"/>
+      <c r="E48" s="38" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="38" t="n"/>
+      <c r="B49" s="38" t="n"/>
+      <c r="C49" s="39" t="n"/>
+      <c r="D49" s="40" t="n"/>
+      <c r="E49" s="38" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="38" t="n"/>
+      <c r="B50" s="38" t="n"/>
+      <c r="C50" s="39" t="n"/>
+      <c r="D50" s="40" t="n"/>
+      <c r="E50" s="38" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="38" t="n"/>
+      <c r="B51" s="38" t="n"/>
+      <c r="C51" s="39" t="n"/>
+      <c r="D51" s="40" t="n"/>
+      <c r="E51" s="38" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="38" t="n"/>
+      <c r="B52" s="38" t="n"/>
+      <c r="C52" s="39" t="n"/>
+      <c r="D52" s="40" t="n"/>
+      <c r="E52" s="38" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="38" t="n"/>
+      <c r="B53" s="38" t="n"/>
+      <c r="C53" s="39" t="n"/>
+      <c r="D53" s="40" t="n"/>
+      <c r="E53" s="38" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="38" t="n"/>
+      <c r="B54" s="38" t="n"/>
+      <c r="C54" s="39" t="n"/>
+      <c r="D54" s="40" t="n"/>
+      <c r="E54" s="38" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="38" t="n"/>
+      <c r="B55" s="38" t="n"/>
+      <c r="C55" s="39" t="n"/>
+      <c r="D55" s="40" t="n"/>
+      <c r="E55" s="38" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="38" t="n"/>
+      <c r="B56" s="38" t="n"/>
+      <c r="C56" s="39" t="n"/>
+      <c r="D56" s="40" t="n"/>
+      <c r="E56" s="38" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="38" t="n"/>
+      <c r="B57" s="38" t="n"/>
+      <c r="C57" s="39" t="n"/>
+      <c r="D57" s="40" t="n"/>
+      <c r="E57" s="38" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="38" t="n"/>
+      <c r="B58" s="38" t="n"/>
+      <c r="C58" s="39" t="n"/>
+      <c r="D58" s="40" t="n"/>
+      <c r="E58" s="38" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="38" t="n"/>
+      <c r="B59" s="38" t="n"/>
+      <c r="C59" s="39" t="n"/>
+      <c r="D59" s="40" t="n"/>
+      <c r="E59" s="38" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="38" t="n"/>
+      <c r="B60" s="38" t="n"/>
+      <c r="C60" s="39" t="n"/>
+      <c r="D60" s="40" t="n"/>
+      <c r="E60" s="38" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="38" t="n"/>
+      <c r="B61" s="38" t="n"/>
+      <c r="C61" s="39" t="n"/>
+      <c r="D61" s="40" t="n"/>
+      <c r="E61" s="38" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="38" t="n"/>
+      <c r="B62" s="38" t="n"/>
+      <c r="C62" s="39" t="n"/>
+      <c r="D62" s="40" t="n"/>
+      <c r="E62" s="38" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="38" t="n"/>
+      <c r="B63" s="38" t="n"/>
+      <c r="C63" s="39" t="n"/>
+      <c r="D63" s="40" t="n"/>
+      <c r="E63" s="38" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="38" t="n"/>
+      <c r="B64" s="38" t="n"/>
+      <c r="C64" s="39" t="n"/>
+      <c r="D64" s="40" t="n"/>
+      <c r="E64" s="38" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="38" t="n"/>
+      <c r="B65" s="38" t="n"/>
+      <c r="C65" s="39" t="n"/>
+      <c r="D65" s="40" t="n"/>
+      <c r="E65" s="38" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="38" t="n"/>
+      <c r="B66" s="38" t="n"/>
+      <c r="C66" s="39" t="n"/>
+      <c r="D66" s="40" t="n"/>
+      <c r="E66" s="38" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="38" t="n"/>
+      <c r="B67" s="38" t="n"/>
+      <c r="C67" s="39" t="n"/>
+      <c r="D67" s="40" t="n"/>
+      <c r="E67" s="38" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="38" t="n"/>
+      <c r="B68" s="38" t="n"/>
+      <c r="C68" s="39" t="n"/>
+      <c r="D68" s="40" t="n"/>
+      <c r="E68" s="38" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="38" t="n"/>
+      <c r="B69" s="38" t="n"/>
+      <c r="C69" s="39" t="n"/>
+      <c r="D69" s="40" t="n"/>
+      <c r="E69" s="38" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="38" t="n"/>
+      <c r="B70" s="38" t="n"/>
+      <c r="C70" s="39" t="n"/>
+      <c r="D70" s="40" t="n"/>
+      <c r="E70" s="38" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="38" t="n"/>
+      <c r="B71" s="38" t="n"/>
+      <c r="C71" s="39" t="n"/>
+      <c r="D71" s="40" t="n"/>
+      <c r="E71" s="38" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="38" t="n"/>
+      <c r="B72" s="38" t="n"/>
+      <c r="C72" s="39" t="n"/>
+      <c r="D72" s="40" t="n"/>
+      <c r="E72" s="38" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="38" t="n"/>
+      <c r="B73" s="38" t="n"/>
+      <c r="C73" s="39" t="n"/>
+      <c r="D73" s="40" t="n"/>
+      <c r="E73" s="38" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="38" t="n"/>
+      <c r="B74" s="38" t="n"/>
+      <c r="C74" s="39" t="n"/>
+      <c r="D74" s="40" t="n"/>
+      <c r="E74" s="38" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="38" t="n"/>
+      <c r="B75" s="38" t="n"/>
+      <c r="C75" s="39" t="n"/>
+      <c r="D75" s="40" t="n"/>
+      <c r="E75" s="38" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="38" t="n"/>
+      <c r="B76" s="38" t="n"/>
+      <c r="C76" s="39" t="n"/>
+      <c r="D76" s="40" t="n"/>
+      <c r="E76" s="38" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="38" t="n"/>
+      <c r="B77" s="38" t="n"/>
+      <c r="C77" s="39" t="n"/>
+      <c r="D77" s="40" t="n"/>
+      <c r="E77" s="38" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="38" t="n"/>
+      <c r="B78" s="38" t="n"/>
+      <c r="C78" s="39" t="n"/>
+      <c r="D78" s="40" t="n"/>
+      <c r="E78" s="38" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="38" t="n"/>
+      <c r="B79" s="38" t="n"/>
+      <c r="C79" s="39" t="n"/>
+      <c r="D79" s="40" t="n"/>
+      <c r="E79" s="38" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="38" t="n"/>
+      <c r="B80" s="38" t="n"/>
+      <c r="C80" s="39" t="n"/>
+      <c r="D80" s="40" t="n"/>
+      <c r="E80" s="38" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="38" t="n"/>
+      <c r="B81" s="38" t="n"/>
+      <c r="C81" s="39" t="n"/>
+      <c r="D81" s="40" t="n"/>
+      <c r="E81" s="38" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="38" t="n"/>
+      <c r="B82" s="38" t="n"/>
+      <c r="C82" s="39" t="n"/>
+      <c r="D82" s="40" t="n"/>
+      <c r="E82" s="38" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="38" t="n"/>
+      <c r="B83" s="38" t="n"/>
+      <c r="C83" s="39" t="n"/>
+      <c r="D83" s="40" t="n"/>
+      <c r="E83" s="38" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="38" t="n"/>
+      <c r="B84" s="38" t="n"/>
+      <c r="C84" s="39" t="n"/>
+      <c r="D84" s="40" t="n"/>
+      <c r="E84" s="38" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="38" t="n"/>
+      <c r="B85" s="38" t="n"/>
+      <c r="C85" s="39" t="n"/>
+      <c r="D85" s="40" t="n"/>
+      <c r="E85" s="38" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="38" t="n"/>
+      <c r="B86" s="38" t="n"/>
+      <c r="C86" s="39" t="n"/>
+      <c r="D86" s="40" t="n"/>
+      <c r="E86" s="38" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="38" t="n"/>
+      <c r="B87" s="38" t="n"/>
+      <c r="C87" s="39" t="n"/>
+      <c r="D87" s="40" t="n"/>
+      <c r="E87" s="38" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="38" t="n"/>
+      <c r="B88" s="38" t="n"/>
+      <c r="C88" s="39" t="n"/>
+      <c r="D88" s="40" t="n"/>
+      <c r="E88" s="38" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="38" t="n"/>
+      <c r="B89" s="38" t="n"/>
+      <c r="C89" s="39" t="n"/>
+      <c r="D89" s="40" t="n"/>
+      <c r="E89" s="38" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="38" t="n"/>
+      <c r="B90" s="38" t="n"/>
+      <c r="C90" s="39" t="n"/>
+      <c r="D90" s="40" t="n"/>
+      <c r="E90" s="38" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="38" t="n"/>
+      <c r="B91" s="38" t="n"/>
+      <c r="C91" s="39" t="n"/>
+      <c r="D91" s="40" t="n"/>
+      <c r="E91" s="38" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="38" t="n"/>
+      <c r="B92" s="38" t="n"/>
+      <c r="C92" s="39" t="n"/>
+      <c r="D92" s="40" t="n"/>
+      <c r="E92" s="38" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="38" t="n"/>
+      <c r="B93" s="38" t="n"/>
+      <c r="C93" s="39" t="n"/>
+      <c r="D93" s="40" t="n"/>
+      <c r="E93" s="38" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="38" t="n"/>
+      <c r="B94" s="38" t="n"/>
+      <c r="C94" s="39" t="n"/>
+      <c r="D94" s="40" t="n"/>
+      <c r="E94" s="38" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="38" t="n"/>
+      <c r="B95" s="38" t="n"/>
+      <c r="C95" s="39" t="n"/>
+      <c r="D95" s="40" t="n"/>
+      <c r="E95" s="38" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="38" t="n"/>
+      <c r="B96" s="38" t="n"/>
+      <c r="C96" s="39" t="n"/>
+      <c r="D96" s="40" t="n"/>
+      <c r="E96" s="38" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="38" t="n"/>
+      <c r="B97" s="38" t="n"/>
+      <c r="C97" s="39" t="n"/>
+      <c r="D97" s="40" t="n"/>
+      <c r="E97" s="38" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="38" t="n"/>
+      <c r="B98" s="38" t="n"/>
+      <c r="C98" s="39" t="n"/>
+      <c r="D98" s="40" t="n"/>
+      <c r="E98" s="38" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="38" t="n"/>
+      <c r="B99" s="38" t="n"/>
+      <c r="C99" s="39" t="n"/>
+      <c r="D99" s="40" t="n"/>
+      <c r="E99" s="38" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="38" t="n"/>
+      <c r="B100" s="38" t="n"/>
+      <c r="C100" s="39" t="n"/>
+      <c r="D100" s="40" t="n"/>
+      <c r="E100" s="38" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="38" t="n"/>
+      <c r="B101" s="38" t="n"/>
+      <c r="C101" s="39" t="n"/>
+      <c r="D101" s="40" t="n"/>
+      <c r="E101" s="38" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="38" t="n"/>
+      <c r="B102" s="38" t="n"/>
+      <c r="C102" s="39" t="n"/>
+      <c r="D102" s="40" t="n"/>
+      <c r="E102" s="38" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="38" t="n"/>
+      <c r="B103" s="38" t="n"/>
+      <c r="C103" s="39" t="n"/>
+      <c r="D103" s="40" t="n"/>
+      <c r="E103" s="38" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="38" t="n"/>
+      <c r="B104" s="38" t="n"/>
+      <c r="C104" s="39" t="n"/>
+      <c r="D104" s="40" t="n"/>
+      <c r="E104" s="38" t="n"/>
+    </row>
+  </sheetData>
+  <dataValidations count="2">
+    <dataValidation sqref="B5:B500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"5,4,3,2,1"</formula1>
+    </dataValidation>
+    <dataValidation sqref="E5:E500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Sí,No"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>